<commit_message>
Fully linked frontend and backend
</commit_message>
<xml_diff>
--- a/backend/my_products.xlsx
+++ b/backend/my_products.xlsx
@@ -492,7 +492,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BAR-687ED6C03C</t>
+          <t>BAR-4A3B619A78</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -543,7 +543,7 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BAR-F358AD76E8</t>
+          <t>BAR-0FA006B52C</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -594,7 +594,7 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BAR-D38E76687A</t>
+          <t>BAR-12834879F1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>